<commit_message>
Web Tech Assignment 1  & 2
</commit_message>
<xml_diff>
--- a/Assignment/SQL/Assignment6/Assignment6.xlsx
+++ b/Assignment/SQL/Assignment6/Assignment6.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="34">
   <si>
     <t xml:space="preserve">ClientNo</t>
   </si>
@@ -123,10 +123,7 @@
     <t xml:space="preserve">ClientNo (PK)</t>
   </si>
   <si>
-    <t xml:space="preserve">ClientNo (FK)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PropertyNo (FK)</t>
+    <t xml:space="preserve">PropertyNo (PK)</t>
   </si>
 </sst>
 </file>
@@ -203,20 +200,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -415,185 +416,185 @@
   <dimension ref="A1:I6"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15.65"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13.37"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="13.01"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="10.92"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15.65"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="13.01"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="10.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.28"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="0" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="0" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="0" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="0" t="n">
+      <c r="G2" s="1" t="n">
         <v>350</v>
       </c>
-      <c r="H2" s="0" t="s">
+      <c r="H2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="0" t="s">
+      <c r="I2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="0" t="s">
+      <c r="D3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G3" s="0" t="n">
+      <c r="G3" s="1" t="n">
         <v>450</v>
       </c>
-      <c r="H3" s="0" t="s">
+      <c r="H3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="0" t="s">
+      <c r="I3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="0" t="s">
+      <c r="D4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="G4" s="0" t="n">
+      <c r="G4" s="1" t="n">
         <v>350</v>
       </c>
-      <c r="H4" s="0" t="s">
+      <c r="H4" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="I4" s="0" t="s">
+      <c r="I4" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D5" s="0" t="s">
+      <c r="D5" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="G5" s="0" t="n">
+      <c r="G5" s="1" t="n">
         <v>370</v>
       </c>
-      <c r="H5" s="0" t="s">
+      <c r="H5" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I5" s="0" t="s">
+      <c r="I5" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="0" t="s">
+      <c r="D6" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G6" s="0" t="n">
+      <c r="G6" s="1" t="n">
         <v>450</v>
       </c>
-      <c r="H6" s="0" t="s">
+      <c r="H6" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="I6" s="0" t="s">
+      <c r="I6" s="1" t="s">
         <v>21</v>
       </c>
     </row>
@@ -616,184 +617,184 @@
   <dimension ref="A1:E20"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14.47"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="28.57"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="14.56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.47"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="28.57"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="14.56"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D7" s="0" t="s">
+      <c r="D7" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="0" t="n">
+      <c r="C8" s="1" t="n">
         <v>350</v>
       </c>
-      <c r="D8" s="0" t="s">
+      <c r="D8" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="0" t="n">
+      <c r="C9" s="1" t="n">
         <v>450</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C10" s="0" t="n">
+      <c r="C10" s="1" t="n">
         <v>370</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="D15" s="0" t="s">
+      <c r="D15" s="1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C16" s="0" t="s">
+      <c r="C16" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D16" s="0" t="s">
+      <c r="D16" s="1" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="0" t="s">
+      <c r="C17" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D17" s="0" t="s">
+      <c r="D17" s="1" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="C18" s="0" t="s">
+      <c r="C18" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D18" s="0" t="s">
+      <c r="D18" s="1" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="C19" s="0" t="s">
+      <c r="C19" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="D19" s="0" t="s">
+      <c r="D19" s="1" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C20" s="0" t="s">
+      <c r="C20" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="D20" s="0" t="s">
+      <c r="D20" s="1" t="s">
         <v>31</v>
       </c>
     </row>
@@ -816,197 +817,197 @@
   <dimension ref="A1:D26"/>
   <sheetFormatPr defaultColWidth="8.453125" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="21.66"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="23.48"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="23.75"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="10.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="21.66"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="23.48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="23.75"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="0" t="s">
+      <c r="D9" s="1" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="C10" s="0" t="n">
+      <c r="C10" s="1" t="n">
         <v>350</v>
       </c>
-      <c r="D10" s="0" t="s">
+      <c r="D10" s="1" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="0" t="n">
+      <c r="C11" s="1" t="n">
         <v>450</v>
       </c>
-      <c r="D11" s="0" t="s">
+      <c r="D11" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="0" t="n">
+      <c r="C12" s="1" t="n">
         <v>370</v>
       </c>
-      <c r="D12" s="0" t="s">
+      <c r="D12" s="1" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="1" t="s">
+      <c r="A16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="2" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+      <c r="A17" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="2" t="s">
+      <c r="A18" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="3" t="s">
         <v>23</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="1" t="s">
+      <c r="A21" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B21" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="2" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+      <c r="A22" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C22" s="3" t="n">
+      <c r="C22" s="4" t="n">
         <v>36678</v>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" s="4" t="n">
         <v>37134</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="A23" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C23" s="3" t="n">
+      <c r="C23" s="4" t="n">
         <v>37500</v>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" s="4" t="n">
         <v>37500</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C24" s="3" t="n">
+      <c r="C24" s="4" t="n">
         <v>36404</v>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" s="4" t="n">
         <v>36687</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="C25" s="3" t="n">
+      <c r="C25" s="4" t="n">
         <v>36809</v>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" s="4" t="n">
         <v>37226</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="A26" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C26" s="3" t="n">
+      <c r="C26" s="4" t="n">
         <v>37561</v>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" s="4" t="n">
         <v>37834</v>
       </c>
     </row>

</xml_diff>